<commit_message>
Add percentage-point labels (vs TCG all-in) to exact-basket workbook
Per exact size, CK/MP all-in cost as pp vs the TCGplayer baseline: CK
+24pp (5 cards) -> +5pp (100); MP -3pp -> -18pp. New tab in
exact_basket_data.xlsx.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/exact_basket_data.xlsx
+++ b/output/exact_basket_data.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Exact basket sizes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pct points vs TCG" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="+0%;-0%"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -68,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -76,6 +78,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -830,4 +836,113 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Cards in basket</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Card Kingdom (pp vs TCG)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>ManaPool (pp vs TCG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>-0.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>-0.16</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>pp = all-in cost vs TCGplayer all-in, in percentage points. TCGplayer = 0 baseline.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add pp labels vs Card Kingdom baseline
CK = 0 baseline: TCGplayer -19pp (5 cards) -> -5pp (100); ManaPool ~-22pp
throughout. New 'Pct points vs CK' tab.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfSvnLRd6xKJhXvNadj6Qu
</commit_message>
<xml_diff>
--- a/output/exact_basket_data.xlsx
+++ b/output/exact_basket_data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Exact basket sizes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Pct points vs TCG" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pct points vs CK" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -945,4 +946,113 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Cards in basket</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>TCGplayer (pp vs CK)</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>ManaPool (pp vs CK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>pp = all-in cost vs Card Kingdom all-in, in percentage points. Card Kingdom = 0 baseline.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>